<commit_message>
Subindo atualizações de teste de caso
</commit_message>
<xml_diff>
--- a/documentacao/Testes/Caso de Teste/UC37 - MANTER ESPECIALIDADES.xlsx
+++ b/documentacao/Testes/Caso de Teste/UC37 - MANTER ESPECIALIDADES.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="64" uniqueCount="50">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="78" uniqueCount="52">
   <si>
     <t xml:space="preserve">Caso de Teste</t>
   </si>
@@ -41,6 +41,12 @@
   </si>
   <si>
     <t xml:space="preserve">Observações</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Status v2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Observações v2</t>
   </si>
   <si>
     <t xml:space="preserve">CT01</t>
@@ -282,16 +288,12 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="7">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -498,252 +500,294 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:G17"/>
-  <sheetFormatPr defaultColWidth="32.2421875" defaultRowHeight="15" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <dimension ref="A1:I17"/>
+  <sheetFormatPr defaultColWidth="32.2421875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="29.04"/>
     <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="32.22"/>
-    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="3" min="3" style="2" width="32.24"/>
+    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="32.24"/>
     <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="1020" min="4" style="1" width="32.22"/>
-    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="16380" min="1021" style="2" width="32.24"/>
+    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="16380" min="1021" style="1" width="32.24"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16384" min="16381" style="1" width="11.74"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="3" t="s">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="3" t="s">
+      <c r="B1" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="3" t="s">
+      <c r="C1" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="3" t="s">
+      <c r="D1" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="4" t="s">
+      <c r="E1" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="3" t="s">
+      <c r="F1" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="3" t="s">
+      <c r="G1" s="2" t="s">
         <v>6</v>
       </c>
+      <c r="H1" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" s="2" t="s">
+        <v>8</v>
+      </c>
     </row>
     <row r="2" customFormat="false" ht="52.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="B2" s="6" t="s">
-        <v>8</v>
-      </c>
-      <c r="C2" s="6" t="s">
+      <c r="A2" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="D2" s="6" t="s">
+      <c r="B2" s="5" t="s">
         <v>10</v>
       </c>
+      <c r="C2" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="D2" s="5" t="s">
+        <v>12</v>
+      </c>
       <c r="F2" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="H2" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="52.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="B3" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="C3" s="5" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="3" customFormat="false" ht="52.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="5" t="s">
-        <v>12</v>
-      </c>
-      <c r="B3" s="6" t="s">
-        <v>13</v>
-      </c>
-      <c r="C3" s="6" t="s">
-        <v>9</v>
-      </c>
-      <c r="D3" s="6" t="s">
-        <v>14</v>
+      <c r="D3" s="5" t="s">
+        <v>16</v>
       </c>
       <c r="F3" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="H3" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="64.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="B4" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="C4" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="D4" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="F4" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="H4" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="B5" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="C5" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="D5" s="5" t="s">
+        <v>24</v>
+      </c>
+      <c r="F5" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="H5" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="52.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="B6" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="C6" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="D6" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="E6" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="F6" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="H6" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="77.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="B7" s="5" t="s">
+        <v>31</v>
+      </c>
+      <c r="C7" s="5" t="s">
+        <v>32</v>
+      </c>
+      <c r="D7" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="F7" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="H7" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="64.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="B8" s="5" t="s">
+        <v>35</v>
+      </c>
+      <c r="C8" s="5" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="4" customFormat="false" ht="64.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="5" t="s">
-        <v>15</v>
-      </c>
-      <c r="B4" s="6" t="s">
-        <v>16</v>
-      </c>
-      <c r="C4" s="6" t="s">
-        <v>17</v>
-      </c>
-      <c r="D4" s="6" t="s">
-        <v>18</v>
-      </c>
-      <c r="F4" s="1" t="s">
+      <c r="D8" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="F8" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="H8" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="52.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="4" t="s">
+        <v>37</v>
+      </c>
+      <c r="B9" s="5" t="s">
+        <v>38</v>
+      </c>
+      <c r="C9" s="5" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="5" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="5" t="s">
-        <v>19</v>
-      </c>
-      <c r="B5" s="6" t="s">
-        <v>20</v>
-      </c>
-      <c r="C5" s="6" t="s">
-        <v>21</v>
-      </c>
-      <c r="D5" s="6" t="s">
-        <v>22</v>
-      </c>
-      <c r="F5" s="1" t="s">
+      <c r="D9" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="F9" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="H9" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="64.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="B10" s="5" t="s">
+        <v>41</v>
+      </c>
+      <c r="C10" s="5" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="6" customFormat="false" ht="52.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="5" t="s">
-        <v>23</v>
-      </c>
-      <c r="B6" s="6" t="s">
-        <v>24</v>
-      </c>
-      <c r="C6" s="6" t="s">
-        <v>25</v>
-      </c>
-      <c r="D6" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="E6" s="1" t="s">
-        <v>27</v>
-      </c>
-      <c r="F6" s="1" t="s">
+      <c r="D10" s="5" t="s">
+        <v>42</v>
+      </c>
+      <c r="E10" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="F10" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="H10" s="1" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="52.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="4" t="s">
+        <v>45</v>
+      </c>
+      <c r="B11" s="5" t="s">
+        <v>46</v>
+      </c>
+      <c r="C11" s="5" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="7" customFormat="false" ht="77.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="5" t="s">
-        <v>28</v>
-      </c>
-      <c r="B7" s="6" t="s">
-        <v>29</v>
-      </c>
-      <c r="C7" s="6" t="s">
-        <v>30</v>
-      </c>
-      <c r="D7" s="6" t="s">
-        <v>31</v>
-      </c>
-      <c r="F7" s="1" t="s">
+      <c r="D11" s="5" t="s">
+        <v>47</v>
+      </c>
+      <c r="F11" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="H11" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="4" t="s">
+        <v>48</v>
+      </c>
+      <c r="B12" s="5" t="s">
+        <v>49</v>
+      </c>
+      <c r="C12" s="5" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="8" customFormat="false" ht="64.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="5" t="s">
-        <v>32</v>
-      </c>
-      <c r="B8" s="6" t="s">
-        <v>33</v>
-      </c>
-      <c r="C8" s="6" t="s">
-        <v>9</v>
-      </c>
-      <c r="D8" s="6" t="s">
-        <v>34</v>
-      </c>
-      <c r="F8" s="1" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="9" customFormat="false" ht="52.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="5" t="s">
-        <v>35</v>
-      </c>
-      <c r="B9" s="6" t="s">
-        <v>36</v>
-      </c>
-      <c r="C9" s="6" t="s">
-        <v>9</v>
-      </c>
-      <c r="D9" s="6" t="s">
-        <v>37</v>
-      </c>
-      <c r="F9" s="1" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="10" customFormat="false" ht="64.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="5" t="s">
-        <v>38</v>
-      </c>
-      <c r="B10" s="6" t="s">
-        <v>39</v>
-      </c>
-      <c r="C10" s="6" t="s">
-        <v>9</v>
-      </c>
-      <c r="D10" s="6" t="s">
-        <v>40</v>
-      </c>
-      <c r="E10" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="F10" s="1" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="11" customFormat="false" ht="52.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="5" t="s">
-        <v>43</v>
-      </c>
-      <c r="B11" s="6" t="s">
-        <v>44</v>
-      </c>
-      <c r="C11" s="6" t="s">
-        <v>9</v>
-      </c>
-      <c r="D11" s="6" t="s">
-        <v>45</v>
-      </c>
-      <c r="F11" s="1" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="12" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="5" t="s">
-        <v>46</v>
-      </c>
-      <c r="B12" s="6" t="s">
-        <v>47</v>
-      </c>
-      <c r="C12" s="6" t="s">
-        <v>9</v>
-      </c>
-      <c r="D12" s="6" t="s">
-        <v>48</v>
+      <c r="D12" s="5" t="s">
+        <v>50</v>
       </c>
       <c r="E12" s="1" t="s">
-        <v>49</v>
+        <v>51</v>
+      </c>
+      <c r="F12" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="H12" s="1" t="s">
+        <v>13</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="5"/>
-      <c r="B13" s="6"/>
+      <c r="A13" s="4"/>
+      <c r="B13" s="5"/>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="5"/>
-      <c r="B14" s="6"/>
+      <c r="A14" s="4"/>
+      <c r="B14" s="5"/>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="5"/>
-      <c r="B15" s="6"/>
+      <c r="A15" s="4"/>
+      <c r="B15" s="5"/>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="5"/>
-      <c r="B16" s="6"/>
+      <c r="A16" s="4"/>
+      <c r="B16" s="5"/>
     </row>
     <row r="17" customFormat="false" ht="18.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="7"/>
-      <c r="B17" s="7"/>
+      <c r="A17" s="6"/>
+      <c r="B17" s="6"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>

</xml_diff>